<commit_message>
august 2026 new haddock model
</commit_message>
<xml_diff>
--- a/data/00_metadata/sequencing_metadata.xlsx
+++ b/data/00_metadata/sequencing_metadata.xlsx
@@ -355,10 +355,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC141"/>
+  <dimension ref="A1:AQ141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
+    <col min="33" max="33" width="20.7109375" style="2" customWidth="1"/>
+    <col min="37" max="37" width="20.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -494,15 +496,85 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Cruise Id</t>
+          <t>Cruise</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>INVESTIGATOR</t>
+          <t>Station</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Stock Area</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Length String</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Length Value</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Sex</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Sample Date</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Aged By</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Omit Age</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Age Comment</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Age Date</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Tray ID</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Tray Barcode</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Tray Cell</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Tray Comment</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Age Barcode</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>sampling_season</t>
         </is>
@@ -589,7 +661,7 @@
       <c r="Z2">
         <v>0.65</v>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -676,7 +748,7 @@
       <c r="Z3">
         <v>0.65</v>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AQ3" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -763,7 +835,7 @@
       <c r="Z4">
         <v>6.65</v>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AQ4" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -850,7 +922,7 @@
       <c r="Z5">
         <v>3.65</v>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AQ5" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -937,7 +1009,7 @@
       <c r="Z6">
         <v>2.65</v>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AQ6" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1024,7 +1096,7 @@
       <c r="Z7">
         <v>0.65</v>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AQ7" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1111,7 +1183,7 @@
       <c r="Z8">
         <v>2.65</v>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AQ8" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1198,7 +1270,7 @@
       <c r="Z9">
         <v>9.65</v>
       </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AQ9" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1285,7 +1357,7 @@
       <c r="Z10">
         <v>5.65</v>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AQ10" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1372,7 +1444,7 @@
       <c r="Z11">
         <v>1.65</v>
       </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AQ11" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1459,7 +1531,7 @@
       <c r="Z12">
         <v>4.65</v>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AQ12" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1546,7 +1618,7 @@
       <c r="Z13">
         <v>9.65</v>
       </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AQ13" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1633,7 +1705,7 @@
       <c r="Z14">
         <v>0.65</v>
       </c>
-      <c r="AC14" t="inlineStr">
+      <c r="AQ14" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1720,7 +1792,7 @@
       <c r="Z15">
         <v>1.65</v>
       </c>
-      <c r="AC15" t="inlineStr">
+      <c r="AQ15" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1807,7 +1879,7 @@
       <c r="Z16">
         <v>6.65</v>
       </c>
-      <c r="AC16" t="inlineStr">
+      <c r="AQ16" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1894,7 +1966,7 @@
       <c r="Z17">
         <v>7.65</v>
       </c>
-      <c r="AC17" t="inlineStr">
+      <c r="AQ17" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -1981,7 +2053,7 @@
       <c r="Z18">
         <v>6.65</v>
       </c>
-      <c r="AC18" t="inlineStr">
+      <c r="AQ18" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2068,7 +2140,7 @@
       <c r="Z19">
         <v>4.65</v>
       </c>
-      <c r="AC19" t="inlineStr">
+      <c r="AQ19" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2155,7 +2227,7 @@
       <c r="Z20">
         <v>3.65</v>
       </c>
-      <c r="AC20" t="inlineStr">
+      <c r="AQ20" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2242,7 +2314,7 @@
       <c r="Z21">
         <v>4.65</v>
       </c>
-      <c r="AC21" t="inlineStr">
+      <c r="AQ21" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2329,7 +2401,7 @@
       <c r="Z22">
         <v>9.65</v>
       </c>
-      <c r="AC22" t="inlineStr">
+      <c r="AQ22" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2416,7 +2488,7 @@
       <c r="Z23">
         <v>2.65</v>
       </c>
-      <c r="AC23" t="inlineStr">
+      <c r="AQ23" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2503,7 +2575,7 @@
       <c r="Z24">
         <v>7.65</v>
       </c>
-      <c r="AC24" t="inlineStr">
+      <c r="AQ24" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2590,7 +2662,7 @@
       <c r="Z25">
         <v>6.65</v>
       </c>
-      <c r="AC25" t="inlineStr">
+      <c r="AQ25" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2677,7 +2749,7 @@
       <c r="Z26">
         <v>2.65</v>
       </c>
-      <c r="AC26" t="inlineStr">
+      <c r="AQ26" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2764,7 +2836,7 @@
       <c r="Z27">
         <v>1.65</v>
       </c>
-      <c r="AC27" t="inlineStr">
+      <c r="AQ27" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2851,7 +2923,7 @@
       <c r="Z28">
         <v>2.65</v>
       </c>
-      <c r="AC28" t="inlineStr">
+      <c r="AQ28" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -2938,7 +3010,7 @@
       <c r="Z29">
         <v>1.65</v>
       </c>
-      <c r="AC29" t="inlineStr">
+      <c r="AQ29" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3025,7 +3097,7 @@
       <c r="Z30">
         <v>1.65</v>
       </c>
-      <c r="AC30" t="inlineStr">
+      <c r="AQ30" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3112,7 +3184,7 @@
       <c r="Z31">
         <v>6.65</v>
       </c>
-      <c r="AC31" t="inlineStr">
+      <c r="AQ31" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3199,7 +3271,7 @@
       <c r="Z32">
         <v>2.65</v>
       </c>
-      <c r="AC32" t="inlineStr">
+      <c r="AQ32" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3286,7 +3358,7 @@
       <c r="Z33">
         <v>9.65</v>
       </c>
-      <c r="AC33" t="inlineStr">
+      <c r="AQ33" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3373,7 +3445,7 @@
       <c r="Z34">
         <v>7.65</v>
       </c>
-      <c r="AC34" t="inlineStr">
+      <c r="AQ34" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3460,7 +3532,7 @@
       <c r="Z35">
         <v>9.65</v>
       </c>
-      <c r="AC35" t="inlineStr">
+      <c r="AQ35" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3547,7 +3619,7 @@
       <c r="Z36">
         <v>5.65</v>
       </c>
-      <c r="AC36" t="inlineStr">
+      <c r="AQ36" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3634,7 +3706,7 @@
       <c r="Z37">
         <v>3.65</v>
       </c>
-      <c r="AC37" t="inlineStr">
+      <c r="AQ37" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3721,7 +3793,7 @@
       <c r="Z38">
         <v>4.65</v>
       </c>
-      <c r="AC38" t="inlineStr">
+      <c r="AQ38" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3808,7 +3880,7 @@
       <c r="Z39">
         <v>3.65</v>
       </c>
-      <c r="AC39" t="inlineStr">
+      <c r="AQ39" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3895,7 +3967,7 @@
       <c r="Z40">
         <v>6.65</v>
       </c>
-      <c r="AC40" t="inlineStr">
+      <c r="AQ40" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -3982,7 +4054,7 @@
       <c r="Z41">
         <v>0.65</v>
       </c>
-      <c r="AC41" t="inlineStr">
+      <c r="AQ41" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -4069,7 +4141,7 @@
       <c r="Z42">
         <v>0.65</v>
       </c>
-      <c r="AC42" t="inlineStr">
+      <c r="AQ42" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -4171,7 +4243,7 @@
       <c r="Z43">
         <v>10.2</v>
       </c>
-      <c r="AC43" t="inlineStr">
+      <c r="AQ43" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4273,7 +4345,7 @@
       <c r="Z44">
         <v>10.2</v>
       </c>
-      <c r="AC44" t="inlineStr">
+      <c r="AQ44" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4375,7 +4447,7 @@
       <c r="Z45">
         <v>7.2</v>
       </c>
-      <c r="AC45" t="inlineStr">
+      <c r="AQ45" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4477,7 +4549,7 @@
       <c r="Z46">
         <v>7.2</v>
       </c>
-      <c r="AC46" t="inlineStr">
+      <c r="AQ46" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4579,7 +4651,7 @@
       <c r="Z47">
         <v>10.2</v>
       </c>
-      <c r="AC47" t="inlineStr">
+      <c r="AQ47" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4681,7 +4753,7 @@
       <c r="Z48">
         <v>10.2</v>
       </c>
-      <c r="AC48" t="inlineStr">
+      <c r="AQ48" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4783,7 +4855,7 @@
       <c r="Z49">
         <v>7.2</v>
       </c>
-      <c r="AC49" t="inlineStr">
+      <c r="AQ49" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4885,7 +4957,7 @@
       <c r="Z50">
         <v>3.2</v>
       </c>
-      <c r="AC50" t="inlineStr">
+      <c r="AQ50" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -4987,7 +5059,7 @@
       <c r="Z51">
         <v>10.2</v>
       </c>
-      <c r="AC51" t="inlineStr">
+      <c r="AQ51" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5089,7 +5161,7 @@
       <c r="Z52">
         <v>3.2</v>
       </c>
-      <c r="AC52" t="inlineStr">
+      <c r="AQ52" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5191,7 +5263,7 @@
       <c r="Z53">
         <v>2.2</v>
       </c>
-      <c r="AC53" t="inlineStr">
+      <c r="AQ53" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5293,7 +5365,7 @@
       <c r="Z54">
         <v>9.199999999999999</v>
       </c>
-      <c r="AC54" t="inlineStr">
+      <c r="AQ54" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5395,7 +5467,7 @@
       <c r="Z55">
         <v>4.2</v>
       </c>
-      <c r="AC55" t="inlineStr">
+      <c r="AQ55" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5497,7 +5569,7 @@
       <c r="Z56">
         <v>2.2</v>
       </c>
-      <c r="AC56" t="inlineStr">
+      <c r="AQ56" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5599,7 +5671,7 @@
       <c r="Z57">
         <v>3.2</v>
       </c>
-      <c r="AC57" t="inlineStr">
+      <c r="AQ57" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5701,7 +5773,7 @@
       <c r="Z58">
         <v>2.2</v>
       </c>
-      <c r="AC58" t="inlineStr">
+      <c r="AQ58" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5803,7 +5875,7 @@
       <c r="Z59">
         <v>3.2</v>
       </c>
-      <c r="AC59" t="inlineStr">
+      <c r="AQ59" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -5905,7 +5977,7 @@
       <c r="Z60">
         <v>10.2</v>
       </c>
-      <c r="AC60" t="inlineStr">
+      <c r="AQ60" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6007,7 +6079,7 @@
       <c r="Z61">
         <v>4.2</v>
       </c>
-      <c r="AC61" t="inlineStr">
+      <c r="AQ61" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6109,7 +6181,7 @@
       <c r="Z62">
         <v>5.2</v>
       </c>
-      <c r="AC62" t="inlineStr">
+      <c r="AQ62" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6211,7 +6283,7 @@
       <c r="Z63">
         <v>5.2</v>
       </c>
-      <c r="AC63" t="inlineStr">
+      <c r="AQ63" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6313,7 +6385,7 @@
       <c r="Z64">
         <v>2.2</v>
       </c>
-      <c r="AC64" t="inlineStr">
+      <c r="AQ64" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6415,7 +6487,7 @@
       <c r="Z65">
         <v>5.2</v>
       </c>
-      <c r="AC65" t="inlineStr">
+      <c r="AQ65" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6517,7 +6589,7 @@
       <c r="Z66">
         <v>3.2</v>
       </c>
-      <c r="AC66" t="inlineStr">
+      <c r="AQ66" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6619,7 +6691,7 @@
       <c r="Z67">
         <v>10.2</v>
       </c>
-      <c r="AC67" t="inlineStr">
+      <c r="AQ67" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6721,7 +6793,7 @@
       <c r="Z68">
         <v>7.2</v>
       </c>
-      <c r="AC68" t="inlineStr">
+      <c r="AQ68" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6823,7 +6895,7 @@
       <c r="Z69">
         <v>2.2</v>
       </c>
-      <c r="AC69" t="inlineStr">
+      <c r="AQ69" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -6925,7 +6997,7 @@
       <c r="Z70">
         <v>8.199999999999999</v>
       </c>
-      <c r="AC70" t="inlineStr">
+      <c r="AQ70" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -7027,7 +7099,7 @@
       <c r="Z71">
         <v>1.2</v>
       </c>
-      <c r="AC71" t="inlineStr">
+      <c r="AQ71" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -7114,7 +7186,7 @@
       <c r="Z72">
         <v>0.65</v>
       </c>
-      <c r="AC72" t="inlineStr">
+      <c r="AQ72" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7201,7 +7273,7 @@
       <c r="Z73">
         <v>0.65</v>
       </c>
-      <c r="AC73" t="inlineStr">
+      <c r="AQ73" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7288,7 +7360,7 @@
       <c r="Z74">
         <v>1.65</v>
       </c>
-      <c r="AC74" t="inlineStr">
+      <c r="AQ74" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7375,7 +7447,7 @@
       <c r="Z75">
         <v>4.65</v>
       </c>
-      <c r="AC75" t="inlineStr">
+      <c r="AQ75" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7462,7 +7534,7 @@
       <c r="Z76">
         <v>9.65</v>
       </c>
-      <c r="AC76" t="inlineStr">
+      <c r="AQ76" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7549,7 +7621,7 @@
       <c r="Z77">
         <v>3.65</v>
       </c>
-      <c r="AC77" t="inlineStr">
+      <c r="AQ77" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7636,7 +7708,7 @@
       <c r="Z78">
         <v>6.65</v>
       </c>
-      <c r="AC78" t="inlineStr">
+      <c r="AQ78" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7723,7 +7795,7 @@
       <c r="Z79">
         <v>2.65</v>
       </c>
-      <c r="AC79" t="inlineStr">
+      <c r="AQ79" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7810,7 +7882,7 @@
       <c r="Z80">
         <v>0.65</v>
       </c>
-      <c r="AC80" t="inlineStr">
+      <c r="AQ80" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7897,7 +7969,7 @@
       <c r="Z81">
         <v>1.65</v>
       </c>
-      <c r="AC81" t="inlineStr">
+      <c r="AQ81" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -7984,7 +8056,7 @@
       <c r="Z82">
         <v>9.65</v>
       </c>
-      <c r="AC82" t="inlineStr">
+      <c r="AQ82" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8071,7 +8143,7 @@
       <c r="Z83">
         <v>8.65</v>
       </c>
-      <c r="AC83" t="inlineStr">
+      <c r="AQ83" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8158,7 +8230,7 @@
       <c r="Z84">
         <v>4.65</v>
       </c>
-      <c r="AC84" t="inlineStr">
+      <c r="AQ84" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8245,7 +8317,7 @@
       <c r="Z85">
         <v>6.65</v>
       </c>
-      <c r="AC85" t="inlineStr">
+      <c r="AQ85" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8332,7 +8404,7 @@
       <c r="Z86">
         <v>2.65</v>
       </c>
-      <c r="AC86" t="inlineStr">
+      <c r="AQ86" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8419,7 +8491,7 @@
       <c r="Z87">
         <v>9.65</v>
       </c>
-      <c r="AC87" t="inlineStr">
+      <c r="AQ87" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8506,7 +8578,7 @@
       <c r="Z88">
         <v>4.65</v>
       </c>
-      <c r="AC88" t="inlineStr">
+      <c r="AQ88" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8593,7 +8665,7 @@
       <c r="Z89">
         <v>7.65</v>
       </c>
-      <c r="AC89" t="inlineStr">
+      <c r="AQ89" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8680,7 +8752,7 @@
       <c r="Z90">
         <v>6.65</v>
       </c>
-      <c r="AC90" t="inlineStr">
+      <c r="AQ90" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8767,7 +8839,7 @@
       <c r="Z91">
         <v>9.65</v>
       </c>
-      <c r="AC91" t="inlineStr">
+      <c r="AQ91" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8854,7 +8926,7 @@
       <c r="Z92">
         <v>2.65</v>
       </c>
-      <c r="AC92" t="inlineStr">
+      <c r="AQ92" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -8941,7 +9013,7 @@
       <c r="Z93">
         <v>5.65</v>
       </c>
-      <c r="AC93" t="inlineStr">
+      <c r="AQ93" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9028,7 +9100,7 @@
       <c r="Z94">
         <v>1.65</v>
       </c>
-      <c r="AC94" t="inlineStr">
+      <c r="AQ94" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9115,7 +9187,7 @@
       <c r="Z95">
         <v>1.65</v>
       </c>
-      <c r="AC95" t="inlineStr">
+      <c r="AQ95" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9202,7 +9274,7 @@
       <c r="Z96">
         <v>6.65</v>
       </c>
-      <c r="AC96" t="inlineStr">
+      <c r="AQ96" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9289,7 +9361,7 @@
       <c r="Z97">
         <v>3.65</v>
       </c>
-      <c r="AC97" t="inlineStr">
+      <c r="AQ97" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9376,7 +9448,7 @@
       <c r="Z98">
         <v>2.65</v>
       </c>
-      <c r="AC98" t="inlineStr">
+      <c r="AQ98" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9463,7 +9535,7 @@
       <c r="Z99">
         <v>2.65</v>
       </c>
-      <c r="AC99" t="inlineStr">
+      <c r="AQ99" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9550,7 +9622,7 @@
       <c r="Z100">
         <v>1.65</v>
       </c>
-      <c r="AC100" t="inlineStr">
+      <c r="AQ100" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9637,7 +9709,7 @@
       <c r="Z101">
         <v>6.65</v>
       </c>
-      <c r="AC101" t="inlineStr">
+      <c r="AQ101" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9724,7 +9796,7 @@
       <c r="Z102">
         <v>7.65</v>
       </c>
-      <c r="AC102" t="inlineStr">
+      <c r="AQ102" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9811,7 +9883,7 @@
       <c r="Z103">
         <v>9.65</v>
       </c>
-      <c r="AC103" t="inlineStr">
+      <c r="AQ103" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9898,7 +9970,7 @@
       <c r="Z104">
         <v>1.65</v>
       </c>
-      <c r="AC104" t="inlineStr">
+      <c r="AQ104" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -9985,7 +10057,7 @@
       <c r="Z105">
         <v>4.65</v>
       </c>
-      <c r="AC105" t="inlineStr">
+      <c r="AQ105" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -10072,7 +10144,7 @@
       <c r="Z106">
         <v>7.65</v>
       </c>
-      <c r="AC106" t="inlineStr">
+      <c r="AQ106" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -10159,7 +10231,7 @@
       <c r="Z107">
         <v>3.65</v>
       </c>
-      <c r="AC107" t="inlineStr">
+      <c r="AQ107" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -10246,7 +10318,7 @@
       <c r="Z108">
         <v>0.65</v>
       </c>
-      <c r="AC108" t="inlineStr">
+      <c r="AQ108" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -10333,7 +10405,7 @@
       <c r="Z109">
         <v>9.65</v>
       </c>
-      <c r="AC109" t="inlineStr">
+      <c r="AQ109" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -10420,7 +10492,7 @@
       <c r="Z110">
         <v>0.65</v>
       </c>
-      <c r="AC110" t="inlineStr">
+      <c r="AQ110" t="inlineStr">
         <is>
           <t>Fall 2022</t>
         </is>
@@ -10522,7 +10594,7 @@
       <c r="Z111">
         <v>7.2</v>
       </c>
-      <c r="AC111" t="inlineStr">
+      <c r="AQ111" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -10624,7 +10696,7 @@
       <c r="Z112">
         <v>10.2</v>
       </c>
-      <c r="AC112" t="inlineStr">
+      <c r="AQ112" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -10726,7 +10798,7 @@
       <c r="Z113">
         <v>10.2</v>
       </c>
-      <c r="AC113" t="inlineStr">
+      <c r="AQ113" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -10828,7 +10900,7 @@
       <c r="Z114">
         <v>7.2</v>
       </c>
-      <c r="AC114" t="inlineStr">
+      <c r="AQ114" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -10930,7 +11002,7 @@
       <c r="Z115">
         <v>1.2</v>
       </c>
-      <c r="AC115" t="inlineStr">
+      <c r="AQ115" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11032,7 +11104,7 @@
       <c r="Z116">
         <v>7.2</v>
       </c>
-      <c r="AC116" t="inlineStr">
+      <c r="AQ116" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11134,7 +11206,7 @@
       <c r="Z117">
         <v>5.2</v>
       </c>
-      <c r="AC117" t="inlineStr">
+      <c r="AQ117" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11236,7 +11308,7 @@
       <c r="Z118">
         <v>3.2</v>
       </c>
-      <c r="AC118" t="inlineStr">
+      <c r="AQ118" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11338,7 +11410,7 @@
       <c r="Z119">
         <v>4.2</v>
       </c>
-      <c r="AC119" t="inlineStr">
+      <c r="AQ119" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11440,7 +11512,7 @@
       <c r="Z120">
         <v>3.2</v>
       </c>
-      <c r="AC120" t="inlineStr">
+      <c r="AQ120" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11542,7 +11614,7 @@
       <c r="Z121">
         <v>1.2</v>
       </c>
-      <c r="AC121" t="inlineStr">
+      <c r="AQ121" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11644,7 +11716,7 @@
       <c r="Z122">
         <v>10.2</v>
       </c>
-      <c r="AC122" t="inlineStr">
+      <c r="AQ122" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11746,7 +11818,7 @@
       <c r="Z123">
         <v>2.2</v>
       </c>
-      <c r="AC123" t="inlineStr">
+      <c r="AQ123" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11848,7 +11920,7 @@
       <c r="Z124">
         <v>10.2</v>
       </c>
-      <c r="AC124" t="inlineStr">
+      <c r="AQ124" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -11950,7 +12022,7 @@
       <c r="Z125">
         <v>2.2</v>
       </c>
-      <c r="AC125" t="inlineStr">
+      <c r="AQ125" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12052,7 +12124,7 @@
       <c r="Z126">
         <v>3.2</v>
       </c>
-      <c r="AC126" t="inlineStr">
+      <c r="AQ126" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12154,7 +12226,7 @@
       <c r="Z127">
         <v>2.2</v>
       </c>
-      <c r="AC127" t="inlineStr">
+      <c r="AQ127" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12256,7 +12328,7 @@
       <c r="Z128">
         <v>7.2</v>
       </c>
-      <c r="AC128" t="inlineStr">
+      <c r="AQ128" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12358,7 +12430,7 @@
       <c r="Z129">
         <v>3.2</v>
       </c>
-      <c r="AC129" t="inlineStr">
+      <c r="AQ129" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12460,7 +12532,7 @@
       <c r="Z130">
         <v>4.2</v>
       </c>
-      <c r="AC130" t="inlineStr">
+      <c r="AQ130" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12562,7 +12634,7 @@
       <c r="Z131">
         <v>3.2</v>
       </c>
-      <c r="AC131" t="inlineStr">
+      <c r="AQ131" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12664,7 +12736,7 @@
       <c r="Z132">
         <v>5.2</v>
       </c>
-      <c r="AC132" t="inlineStr">
+      <c r="AQ132" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12766,7 +12838,7 @@
       <c r="Z133">
         <v>6.2</v>
       </c>
-      <c r="AC133" t="inlineStr">
+      <c r="AQ133" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12868,7 +12940,7 @@
       <c r="Z134">
         <v>2.2</v>
       </c>
-      <c r="AC134" t="inlineStr">
+      <c r="AQ134" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -12970,7 +13042,7 @@
       <c r="Z135">
         <v>10.2</v>
       </c>
-      <c r="AC135" t="inlineStr">
+      <c r="AQ135" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -13072,7 +13144,7 @@
       <c r="Z136">
         <v>5.2</v>
       </c>
-      <c r="AC136" t="inlineStr">
+      <c r="AQ136" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -13174,7 +13246,7 @@
       <c r="Z137">
         <v>5.2</v>
       </c>
-      <c r="AC137" t="inlineStr">
+      <c r="AQ137" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -13276,7 +13348,7 @@
       <c r="Z138">
         <v>2.2</v>
       </c>
-      <c r="AC138" t="inlineStr">
+      <c r="AQ138" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -13378,7 +13450,7 @@
       <c r="Z139">
         <v>7.2</v>
       </c>
-      <c r="AC139" t="inlineStr">
+      <c r="AQ139" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -13480,7 +13552,7 @@
       <c r="Z140">
         <v>3.2</v>
       </c>
-      <c r="AC140" t="inlineStr">
+      <c r="AQ140" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>
@@ -13582,7 +13654,7 @@
       <c r="Z141">
         <v>2.2</v>
       </c>
-      <c r="AC141" t="inlineStr">
+      <c r="AQ141" t="inlineStr">
         <is>
           <t>Spring 2023</t>
         </is>

</xml_diff>